<commit_message>
Best Lifter: Proper championships and age groups automatically
</commit_message>
<xml_diff>
--- a/local/templates/competitionBook/BestLifter-NoPlaque.xlsx
+++ b/local/templates/competitionBook/BestLifter-NoPlaque.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Library/Application Support/owlcms/64.0.2+quick-start/local/templates/competitionBook/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Projects/nemikor/usaw-owlcms/local/templates/competitionBook/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{531300B3-F039-6E4E-8929-BB21909331C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5682C637-108C-1242-8F5B-CA0EF0FA12DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1540" yWindow="660" windowWidth="33020" windowHeight="21680" xr2:uid="{C695CBD2-3DAD-B341-8FFD-602D797EB14F}"/>
+    <workbookView xWindow="27360" yWindow="4400" windowWidth="33020" windowHeight="21680" xr2:uid="{C695CBD2-3DAD-B341-8FFD-602D797EB14F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -359,10 +359,10 @@
     <t>${athlete.team}</t>
   </si>
   <si>
-    <t>${mBest.0.ageGroup.championshipName} - Best Lifters</t>
-  </si>
-  <si>
     <t>No Plaque Awarded</t>
+  </si>
+  <si>
+    <t>${ageGroupPrefix ? ageGroupPrefix : championship ? championship.name : ""}${championship ? " - " : ""}Best Lifters</t>
   </si>
 </sst>
 </file>
@@ -925,7 +925,7 @@
     </row>
     <row r="2" spans="1:16" ht="19" x14ac:dyDescent="0.2">
       <c r="A2" s="16" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B2" s="16"/>
       <c r="C2" s="16"/>
@@ -945,7 +945,7 @@
     </row>
     <row r="3" spans="1:16" ht="19" x14ac:dyDescent="0.2">
       <c r="A3" s="16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="16"/>

</xml_diff>

<commit_message>
Best Lifter: Handle athletes out of competition
</commit_message>
<xml_diff>
--- a/local/templates/competitionBook/BestLifter-NoPlaque.xlsx
+++ b/local/templates/competitionBook/BestLifter-NoPlaque.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Projects/nemikor/usaw-owlcms/local/templates/competitionBook/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5682C637-108C-1242-8F5B-CA0EF0FA12DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68758257-2CF6-A547-92AD-29A041DB4772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="27360" yWindow="4400" windowWidth="33020" windowHeight="21680" xr2:uid="{C695CBD2-3DAD-B341-8FFD-602D797EB14F}"/>
   </bookViews>
@@ -50,7 +50,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>jx:area(lastCell="I15")</t>
+          <t>jx:area(lastCell="J15")</t>
         </r>
       </text>
     </comment>
@@ -103,7 +103,7 @@
             <rFont val="Tahoma"/>
             <family val="34"/>
           </rPr>
-          <t xml:space="preserve">  lastCell="I9"
+          <t xml:space="preserve">  lastCell="J9"
 </t>
         </r>
         <r>
@@ -153,7 +153,7 @@
             <rFont val="Tahoma"/>
             <family val="34"/>
           </rPr>
-          <t xml:space="preserve">  lastCell="I9"
+          <t xml:space="preserve">  lastCell="J9"
 </t>
         </r>
         <r>
@@ -216,7 +216,7 @@
             <rFont val="Tahoma"/>
             <family val="34"/>
           </rPr>
-          <t xml:space="preserve">  lastCell="I15"
+          <t xml:space="preserve">  lastCell="J15"
 </t>
         </r>
         <r>
@@ -266,7 +266,7 @@
             <rFont val="Tahoma"/>
             <family val="34"/>
           </rPr>
-          <t xml:space="preserve">  lastCell="I15"
+          <t xml:space="preserve">  lastCell="J15"
 </t>
         </r>
         <r>
@@ -285,7 +285,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="28">
   <si>
     <t>${competition.competitionName}</t>
   </si>
@@ -363,6 +363,12 @@
   </si>
   <si>
     <t>${ageGroupPrefix ? ageGroupPrefix : championship ? championship.name : ""}${championship ? " - " : ""}Best Lifters</t>
+  </si>
+  <si>
+    <t>Rank</t>
+  </si>
+  <si>
+    <t>${athlete.bestLifterRank == -1 ? "ext" : athlete.bestLifterRank}</t>
   </si>
 </sst>
 </file>
@@ -507,7 +513,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -554,6 +560,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -892,18 +901,19 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="3" width="25.83203125" customWidth="1"/>
-    <col min="4" max="4" width="6.83203125" customWidth="1"/>
-    <col min="5" max="5" width="4.83203125" customWidth="1"/>
-    <col min="6" max="8" width="6.83203125" customWidth="1"/>
-    <col min="9" max="9" width="8.33203125" customWidth="1"/>
+    <col min="1" max="1" width="6.83203125" customWidth="1"/>
+    <col min="2" max="2" width="8.83203125" customWidth="1"/>
+    <col min="3" max="4" width="25.83203125" customWidth="1"/>
+    <col min="5" max="5" width="6.83203125" customWidth="1"/>
+    <col min="6" max="6" width="4.83203125" customWidth="1"/>
+    <col min="7" max="9" width="6.83203125" customWidth="1"/>
+    <col min="10" max="10" width="8.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="19" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:17" ht="19" x14ac:dyDescent="0.2">
       <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
@@ -915,15 +925,16 @@
       <c r="G1" s="16"/>
       <c r="H1" s="16"/>
       <c r="I1" s="16"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="17"/>
       <c r="L1" s="10"/>
       <c r="M1" s="10"/>
       <c r="N1" s="10"/>
       <c r="O1" s="10"/>
       <c r="P1" s="10"/>
+      <c r="Q1" s="10"/>
     </row>
-    <row r="2" spans="1:16" ht="19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:17" ht="19" x14ac:dyDescent="0.2">
       <c r="A2" s="16" t="s">
         <v>25</v>
       </c>
@@ -935,15 +946,16 @@
       <c r="G2" s="16"/>
       <c r="H2" s="16"/>
       <c r="I2" s="16"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="10"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="17"/>
       <c r="L2" s="10"/>
       <c r="M2" s="10"/>
       <c r="N2" s="10"/>
       <c r="O2" s="10"/>
       <c r="P2" s="10"/>
+      <c r="Q2" s="10"/>
     </row>
-    <row r="3" spans="1:16" ht="19" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:17" ht="19" x14ac:dyDescent="0.2">
       <c r="A3" s="16" t="s">
         <v>24</v>
       </c>
@@ -955,15 +967,16 @@
       <c r="G3" s="16"/>
       <c r="H3" s="16"/>
       <c r="I3" s="16"/>
-      <c r="J3" s="10"/>
+      <c r="J3" s="16"/>
       <c r="K3" s="10"/>
       <c r="L3" s="10"/>
       <c r="M3" s="10"/>
       <c r="N3" s="10"/>
       <c r="O3" s="10"/>
       <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
     </row>
-    <row r="4" spans="1:16" ht="19" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" ht="19" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -973,15 +986,16 @@
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
-      <c r="J4" s="10"/>
+      <c r="J4" s="1"/>
       <c r="K4" s="10"/>
       <c r="L4" s="10"/>
       <c r="M4" s="10"/>
       <c r="N4" s="10"/>
       <c r="O4" s="10"/>
       <c r="P4" s="10"/>
+      <c r="Q4" s="10"/>
     </row>
-    <row r="5" spans="1:16" s="12" customFormat="1" ht="19" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" s="12" customFormat="1" ht="19" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
         <v>19</v>
       </c>
@@ -993,90 +1007,98 @@
       <c r="G5" s="15"/>
       <c r="H5" s="15"/>
       <c r="I5" s="15"/>
-      <c r="J5" s="11"/>
+      <c r="J5" s="15"/>
       <c r="K5" s="11"/>
       <c r="L5" s="11"/>
       <c r="M5" s="11"/>
       <c r="N5" s="11"/>
       <c r="O5" s="11"/>
       <c r="P5" s="11"/>
+      <c r="Q5" s="11"/>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="3"/>
       <c r="C7" s="3"/>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="3"/>
+      <c r="E7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E7" s="3"/>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="3"/>
+      <c r="G7" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="14"/>
-      <c r="H7" s="3"/>
+      <c r="H7" s="14"/>
       <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="F8" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="G8" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="H8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="I8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="J8" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="C9" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="D9" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="E9" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="F9" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="I9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="J9" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:16" s="12" customFormat="1" ht="19" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17" s="12" customFormat="1" ht="19" x14ac:dyDescent="0.2">
       <c r="A11" s="15" t="s">
         <v>20</v>
       </c>
@@ -1088,98 +1110,106 @@
       <c r="G11" s="15"/>
       <c r="H11" s="15"/>
       <c r="I11" s="15"/>
-      <c r="J11" s="11"/>
+      <c r="J11" s="15"/>
       <c r="K11" s="11"/>
       <c r="L11" s="11"/>
       <c r="M11" s="11"/>
       <c r="N11" s="11"/>
       <c r="O11" s="11"/>
       <c r="P11" s="11"/>
+      <c r="Q11" s="11"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A13" s="3"/>
+      <c r="B13" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B13" s="3"/>
       <c r="C13" s="3"/>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="3"/>
+      <c r="E13" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E13" s="3"/>
-      <c r="F13" s="13" t="s">
+      <c r="F13" s="3"/>
+      <c r="G13" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="G13" s="14"/>
-      <c r="H13" s="3"/>
+      <c r="H13" s="14"/>
       <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="C14" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="E14" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="F14" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="G14" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="H14" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="I14" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="I14" s="4" t="s">
+      <c r="J14" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="C15" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="D15" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="E15" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="F15" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="G15" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="H15" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="I15" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="J15" s="2" t="s">
         <v>18</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A11:I11"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="69" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>